<commit_message>
feat(calculators): tests build and passing for 16.1.1.4
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/16-lulucf/16-lulucf.xlsx
+++ b/packages/calculators/src/modules/test/16-lulucf/16-lulucf.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eddiesholl/Code/aginnovationaustralia/emissions-calculators/packages/calculators/src/modules/test/16-lulucf/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8D5EE67-ED7D-8240-9962-E92121F439EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7E4D61C-54AB-8948-B785-95693C118AF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51220" yWindow="13240" windowWidth="28800" windowHeight="27420" xr2:uid="{CC0FEAF9-C40F-694B-BCB9-117AFB86C05D}"/>
+    <workbookView xWindow="51220" yWindow="13240" windowWidth="28800" windowHeight="27420" activeTab="1" xr2:uid="{CC0FEAF9-C40F-694B-BCB9-117AFB86C05D}"/>
   </bookViews>
   <sheets>
     <sheet name="16.1.1.2" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="134">
   <si>
     <t>Scenario</t>
   </si>
@@ -512,6 +512,12 @@
   </si>
   <si>
     <t>FullCAM</t>
+  </si>
+  <si>
+    <t>Empty</t>
+  </si>
+  <si>
+    <t>Large</t>
   </si>
 </sst>
 </file>
@@ -1154,7 +1160,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92CDB52C-734F-7046-ACDC-C5573D991542}">
-  <dimension ref="A4:D11"/>
+  <dimension ref="A4:D13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="16.1640625" customWidth="1"/>
@@ -1224,6 +1230,36 @@
       <c r="D11">
         <f>B11*C11</f>
         <v>125</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>132</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="D12">
+        <f t="shared" ref="D12:D13" si="0">B12*C12</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>133</v>
+      </c>
+      <c r="B13">
+        <v>35</v>
+      </c>
+      <c r="C13">
+        <v>200</v>
+      </c>
+      <c r="D13">
+        <f t="shared" si="0"/>
+        <v>7000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(calculators): tests built and passing for 16.1.1.5 biomass burning
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/16-lulucf/16-lulucf.xlsx
+++ b/packages/calculators/src/modules/test/16-lulucf/16-lulucf.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eddiesholl/Code/aginnovationaustralia/emissions-calculators/packages/calculators/src/modules/test/16-lulucf/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7E4D61C-54AB-8948-B785-95693C118AF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48E8A84F-F8F7-AB43-905E-4C39A8AD87BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51220" yWindow="13240" windowWidth="28800" windowHeight="27420" activeTab="1" xr2:uid="{CC0FEAF9-C40F-694B-BCB9-117AFB86C05D}"/>
+    <workbookView xWindow="51220" yWindow="13240" windowWidth="28800" windowHeight="27420" activeTab="2" xr2:uid="{CC0FEAF9-C40F-694B-BCB9-117AFB86C05D}"/>
   </bookViews>
   <sheets>
     <sheet name="16.1.1.2" sheetId="1" r:id="rId1"/>
@@ -211,259 +211,7 @@
     <t>aij=1-3y</t>
   </si>
   <si>
-    <t>Arnhem Coast </t>
-  </si>
-  <si>
-    <t>Arnhem Plateau </t>
-  </si>
-  <si>
-    <t>Australian Alps </t>
-  </si>
-  <si>
-    <t>Avon Wheatbelt </t>
-  </si>
-  <si>
-    <t>Brigalow Belt North </t>
-  </si>
-  <si>
-    <t>Brigalow Belt South </t>
-  </si>
-  <si>
-    <t>Ben Lomond </t>
-  </si>
-  <si>
-    <t>Broken Hill Complex </t>
-  </si>
-  <si>
-    <t>Burt Plain </t>
-  </si>
-  <si>
-    <t>Carnarvon </t>
-  </si>
-  <si>
-    <t>Central Arnhem </t>
-  </si>
-  <si>
-    <t>Central Kimberley </t>
-  </si>
-  <si>
-    <t>Central Ranges </t>
-  </si>
-  <si>
-    <t>Channel Country </t>
-  </si>
-  <si>
-    <t>Central Mackay Coast </t>
-  </si>
-  <si>
-    <t>Coolgardie </t>
-  </si>
-  <si>
-    <t>Cobar Peneplain </t>
-  </si>
-  <si>
-    <t>Cape York Peninsula </t>
-  </si>
-  <si>
-    <t>Daly Basin </t>
-  </si>
-  <si>
-    <t>Darwin Coastal </t>
-  </si>
-  <si>
     <t>Region</t>
-  </si>
-  <si>
-    <t>Dampierland </t>
-  </si>
-  <si>
-    <t>Desert Uplands </t>
-  </si>
-  <si>
-    <t>Davenport Murchison Ranges </t>
-  </si>
-  <si>
-    <t>Darling Riverine Plains </t>
-  </si>
-  <si>
-    <t>Einasleigh Uplands </t>
-  </si>
-  <si>
-    <t>Esperance Plains </t>
-  </si>
-  <si>
-    <t>Eyre Yorke Block </t>
-  </si>
-  <si>
-    <t>Flinders Lofty Block </t>
-  </si>
-  <si>
-    <t>Furneaux </t>
-  </si>
-  <si>
-    <t>Gascoyne </t>
-  </si>
-  <si>
-    <t>Gawler </t>
-  </si>
-  <si>
-    <t>Geraldton Sandplains </t>
-  </si>
-  <si>
-    <t>Gulf Fall and Uplands </t>
-  </si>
-  <si>
-    <t>Gibson Desert </t>
-  </si>
-  <si>
-    <t>Great Sandy Desert </t>
-  </si>
-  <si>
-    <t>Gulf Coastal </t>
-  </si>
-  <si>
-    <t>Gulf Plains </t>
-  </si>
-  <si>
-    <t>Great Victoria Desert </t>
-  </si>
-  <si>
-    <t>Hampton </t>
-  </si>
-  <si>
-    <t>Jarrah Forest </t>
-  </si>
-  <si>
-    <t>Kanmantoo </t>
-  </si>
-  <si>
-    <t>King </t>
-  </si>
-  <si>
-    <t>Little Sandy Desert </t>
-  </si>
-  <si>
-    <t>MacDonnell Ranges </t>
-  </si>
-  <si>
-    <t>Mallee </t>
-  </si>
-  <si>
-    <t>Murray Darling Depression </t>
-  </si>
-  <si>
-    <t>Mitchell Grass Downs </t>
-  </si>
-  <si>
-    <t>Mount Isa Inlier </t>
-  </si>
-  <si>
-    <t>Mulga Lands </t>
-  </si>
-  <si>
-    <t>Murchison </t>
-  </si>
-  <si>
-    <t>Nandewar </t>
-  </si>
-  <si>
-    <t>Naracoorte Coastal Plain </t>
-  </si>
-  <si>
-    <t>New England Tablelands </t>
-  </si>
-  <si>
-    <t>NSW North Coast </t>
-  </si>
-  <si>
-    <t>Northern Kimberley </t>
-  </si>
-  <si>
-    <t>NSW South Western Slopes </t>
-  </si>
-  <si>
-    <t>Nullarbor </t>
-  </si>
-  <si>
-    <t>Ord Victoria Plain </t>
-  </si>
-  <si>
-    <t>Pine Creek </t>
-  </si>
-  <si>
-    <t>Pilbara </t>
-  </si>
-  <si>
-    <t>Riverina </t>
-  </si>
-  <si>
-    <t>South East Coastal Plain </t>
-  </si>
-  <si>
-    <t>South East Corner </t>
-  </si>
-  <si>
-    <t>South Eastern Highlands </t>
-  </si>
-  <si>
-    <t>South Eastern Queensland </t>
-  </si>
-  <si>
-    <t>Simpson Strzelecki Dunefields </t>
-  </si>
-  <si>
-    <t>Stony Plains </t>
-  </si>
-  <si>
-    <t>Sturt Plateau </t>
-  </si>
-  <si>
-    <t>Southern Volcanic Plain </t>
-  </si>
-  <si>
-    <t>Swan Coastal Plain </t>
-  </si>
-  <si>
-    <t>Sydney Basin </t>
-  </si>
-  <si>
-    <t>Tanami </t>
-  </si>
-  <si>
-    <t>Tasmanian Central Highlands </t>
-  </si>
-  <si>
-    <t>Tiwi Cobourg </t>
-  </si>
-  <si>
-    <t>Tasmanian Northern Midlands </t>
-  </si>
-  <si>
-    <t>Tasmanian Northern Slopes </t>
-  </si>
-  <si>
-    <t>Tasmanian South East </t>
-  </si>
-  <si>
-    <t>Tasmanian Southern Ranges </t>
-  </si>
-  <si>
-    <t>Tasmanian West </t>
-  </si>
-  <si>
-    <t>Victoria Bonaparte </t>
-  </si>
-  <si>
-    <t>Victorian Midlands </t>
-  </si>
-  <si>
-    <t>Warren </t>
-  </si>
-  <si>
-    <t>Wet Tropics </t>
-  </si>
-  <si>
-    <t>Yalgoo </t>
   </si>
   <si>
     <r>
@@ -518,6 +266,258 @@
   </si>
   <si>
     <t>Large</t>
+  </si>
+  <si>
+    <t>Arnhem Coast</t>
+  </si>
+  <si>
+    <t>Arnhem Plateau</t>
+  </si>
+  <si>
+    <t>Australian Alps</t>
+  </si>
+  <si>
+    <t>Avon Wheatbelt</t>
+  </si>
+  <si>
+    <t>Brigalow Belt North</t>
+  </si>
+  <si>
+    <t>Brigalow Belt South</t>
+  </si>
+  <si>
+    <t>Ben Lomond</t>
+  </si>
+  <si>
+    <t>Broken Hill Complex</t>
+  </si>
+  <si>
+    <t>Burt Plain</t>
+  </si>
+  <si>
+    <t>Carnarvon</t>
+  </si>
+  <si>
+    <t>Central Arnhem</t>
+  </si>
+  <si>
+    <t>Central Kimberley</t>
+  </si>
+  <si>
+    <t>Central Ranges</t>
+  </si>
+  <si>
+    <t>Channel Country</t>
+  </si>
+  <si>
+    <t>Central Mackay Coast</t>
+  </si>
+  <si>
+    <t>Coolgardie</t>
+  </si>
+  <si>
+    <t>Cobar Peneplain</t>
+  </si>
+  <si>
+    <t>Cape York Peninsula</t>
+  </si>
+  <si>
+    <t>Daly Basin</t>
+  </si>
+  <si>
+    <t>Darwin Coastal</t>
+  </si>
+  <si>
+    <t>Dampierland</t>
+  </si>
+  <si>
+    <t>Desert Uplands</t>
+  </si>
+  <si>
+    <t>Davenport Murchison Ranges</t>
+  </si>
+  <si>
+    <t>Darling Riverine Plains</t>
+  </si>
+  <si>
+    <t>Einasleigh Uplands</t>
+  </si>
+  <si>
+    <t>Esperance Plains</t>
+  </si>
+  <si>
+    <t>Eyre Yorke Block</t>
+  </si>
+  <si>
+    <t>Flinders Lofty Block</t>
+  </si>
+  <si>
+    <t>Furneaux</t>
+  </si>
+  <si>
+    <t>Gascoyne</t>
+  </si>
+  <si>
+    <t>Gawler</t>
+  </si>
+  <si>
+    <t>Geraldton Sandplains</t>
+  </si>
+  <si>
+    <t>Gulf Fall and Uplands</t>
+  </si>
+  <si>
+    <t>Gibson Desert</t>
+  </si>
+  <si>
+    <t>Great Sandy Desert</t>
+  </si>
+  <si>
+    <t>Gulf Coastal</t>
+  </si>
+  <si>
+    <t>Gulf Plains</t>
+  </si>
+  <si>
+    <t>Great Victoria Desert</t>
+  </si>
+  <si>
+    <t>Hampton</t>
+  </si>
+  <si>
+    <t>Jarrah Forest</t>
+  </si>
+  <si>
+    <t>Kanmantoo</t>
+  </si>
+  <si>
+    <t>King</t>
+  </si>
+  <si>
+    <t>Little Sandy Desert</t>
+  </si>
+  <si>
+    <t>MacDonnell Ranges</t>
+  </si>
+  <si>
+    <t>Mallee</t>
+  </si>
+  <si>
+    <t>Murray Darling Depression</t>
+  </si>
+  <si>
+    <t>Mitchell Grass Downs</t>
+  </si>
+  <si>
+    <t>Mount Isa Inlier</t>
+  </si>
+  <si>
+    <t>Mulga Lands</t>
+  </si>
+  <si>
+    <t>Murchison</t>
+  </si>
+  <si>
+    <t>Nandewar</t>
+  </si>
+  <si>
+    <t>Naracoorte Coastal Plain</t>
+  </si>
+  <si>
+    <t>New England Tablelands</t>
+  </si>
+  <si>
+    <t>NSW North Coast</t>
+  </si>
+  <si>
+    <t>Northern Kimberley</t>
+  </si>
+  <si>
+    <t>NSW South Western Slopes</t>
+  </si>
+  <si>
+    <t>Nullarbor</t>
+  </si>
+  <si>
+    <t>Ord Victoria Plain</t>
+  </si>
+  <si>
+    <t>Pine Creek</t>
+  </si>
+  <si>
+    <t>Pilbara</t>
+  </si>
+  <si>
+    <t>Riverina</t>
+  </si>
+  <si>
+    <t>South East Coastal Plain</t>
+  </si>
+  <si>
+    <t>South East Corner</t>
+  </si>
+  <si>
+    <t>South Eastern Highlands</t>
+  </si>
+  <si>
+    <t>South Eastern Queensland</t>
+  </si>
+  <si>
+    <t>Simpson Strzelecki Dunefields</t>
+  </si>
+  <si>
+    <t>Stony Plains</t>
+  </si>
+  <si>
+    <t>Sturt Plateau</t>
+  </si>
+  <si>
+    <t>Southern Volcanic Plain</t>
+  </si>
+  <si>
+    <t>Swan Coastal Plain</t>
+  </si>
+  <si>
+    <t>Sydney Basin</t>
+  </si>
+  <si>
+    <t>Tanami</t>
+  </si>
+  <si>
+    <t>Tasmanian Central Highlands</t>
+  </si>
+  <si>
+    <t>Tiwi Cobourg</t>
+  </si>
+  <si>
+    <t>Tasmanian Northern Midlands</t>
+  </si>
+  <si>
+    <t>Tasmanian Northern Slopes</t>
+  </si>
+  <si>
+    <t>Tasmanian South East</t>
+  </si>
+  <si>
+    <t>Tasmanian Southern Ranges</t>
+  </si>
+  <si>
+    <t>Tasmanian West</t>
+  </si>
+  <si>
+    <t>Victoria Bonaparte</t>
+  </si>
+  <si>
+    <t>Victorian Midlands</t>
+  </si>
+  <si>
+    <t>Warren</t>
+  </si>
+  <si>
+    <t>Wet Tropics</t>
+  </si>
+  <si>
+    <t>Yalgoo</t>
   </si>
 </sst>
 </file>
@@ -946,16 +946,16 @@
   <sheetData>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
-        <v>131</v>
+        <v>47</v>
       </c>
       <c r="C4" t="s">
-        <v>131</v>
+        <v>47</v>
       </c>
       <c r="E4" t="s">
-        <v>131</v>
+        <v>47</v>
       </c>
       <c r="F4" t="s">
-        <v>131</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.2">
@@ -1170,7 +1170,7 @@
   <sheetData>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
-        <v>131</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
@@ -1234,7 +1234,7 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>132</v>
+        <v>48</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -1249,7 +1249,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>133</v>
+        <v>49</v>
       </c>
       <c r="B13">
         <v>35</v>
@@ -1314,7 +1314,7 @@
     </row>
     <row r="10" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A10" s="8" t="s">
-        <v>62</v>
+        <v>42</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>41</v>
@@ -1334,7 +1334,7 @@
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="7" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="B11">
         <v>1</v>
@@ -1352,11 +1352,11 @@
         <v>3.67</v>
       </c>
       <c r="F11">
-        <f>D11*E11</f>
-        <v>-0.44039999999999996</v>
+        <f>D11*E11*-1</f>
+        <v>0.44039999999999996</v>
       </c>
       <c r="K11" s="7" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="L11" s="7">
         <v>-0.12</v>
@@ -1364,7 +1364,7 @@
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="7" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B12">
         <v>2</v>
@@ -1382,11 +1382,11 @@
         <v>3.67</v>
       </c>
       <c r="F12">
-        <f t="shared" ref="F12:F75" si="3">D12*E12</f>
-        <v>-2.8626</v>
+        <f t="shared" ref="F12:F75" si="3">D12*E12*-1</f>
+        <v>2.8626</v>
       </c>
       <c r="K12" s="7" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="L12" s="7">
         <v>-0.39</v>
@@ -1394,7 +1394,7 @@
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="B13">
         <v>3</v>
@@ -1413,10 +1413,10 @@
       </c>
       <c r="F13">
         <f t="shared" si="3"/>
-        <v>-0.9909</v>
+        <v>0.9909</v>
       </c>
       <c r="K13" s="7" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="L13" s="7">
         <v>-0.09</v>
@@ -1424,7 +1424,7 @@
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="7" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="B14">
         <v>4</v>
@@ -1443,10 +1443,10 @@
       </c>
       <c r="F14">
         <f t="shared" si="3"/>
-        <v>-1.3211999999999999</v>
+        <v>1.3211999999999999</v>
       </c>
       <c r="K14" s="7" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="L14" s="7">
         <v>-0.09</v>
@@ -1454,7 +1454,7 @@
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="7" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="B15">
         <v>5</v>
@@ -1473,10 +1473,10 @@
       </c>
       <c r="F15">
         <f t="shared" si="3"/>
-        <v>-2.3855</v>
+        <v>2.3855</v>
       </c>
       <c r="K15" s="7" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="L15" s="7">
         <v>-0.13</v>
@@ -1484,7 +1484,7 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="7" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="B16">
         <v>6</v>
@@ -1503,10 +1503,10 @@
       </c>
       <c r="F16">
         <f t="shared" si="3"/>
-        <v>-2.8626</v>
+        <v>2.8626</v>
       </c>
       <c r="K16" s="7" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="L16" s="7">
         <v>-0.13</v>
@@ -1514,7 +1514,7 @@
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" s="7" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="B17">
         <v>7</v>
@@ -1533,10 +1533,10 @@
       </c>
       <c r="F17">
         <f t="shared" si="3"/>
-        <v>-14.129500000000002</v>
+        <v>14.129500000000002</v>
       </c>
       <c r="K17" s="7" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="L17" s="7">
         <v>-0.55000000000000004</v>
@@ -1544,7 +1544,7 @@
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" s="7" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="B18">
         <v>8</v>
@@ -1563,10 +1563,10 @@
       </c>
       <c r="F18">
         <f t="shared" si="3"/>
-        <v>-0.29360000000000003</v>
+        <v>0.29360000000000003</v>
       </c>
       <c r="K18" s="7" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="L18" s="7">
         <v>-0.01</v>
@@ -1574,7 +1574,7 @@
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" s="7" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="B19">
         <v>9</v>
@@ -1593,10 +1593,10 @@
       </c>
       <c r="F19">
         <f t="shared" si="3"/>
-        <v>-2.3121000000000005</v>
+        <v>2.3121000000000005</v>
       </c>
       <c r="K19" s="7" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="L19" s="7">
         <v>-7.0000000000000007E-2</v>
@@ -1604,7 +1604,7 @@
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="B20">
         <v>10</v>
@@ -1623,10 +1623,10 @@
       </c>
       <c r="F20">
         <f t="shared" si="3"/>
-        <v>-2.202</v>
+        <v>2.202</v>
       </c>
       <c r="K20" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="L20" s="7">
         <v>-0.06</v>
@@ -1634,7 +1634,7 @@
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" s="7" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="B21">
         <v>11</v>
@@ -1653,10 +1653,10 @@
       </c>
       <c r="F21">
         <f t="shared" si="3"/>
-        <v>-3.6332999999999998</v>
+        <v>3.6332999999999998</v>
       </c>
       <c r="K21" s="7" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="L21" s="7">
         <v>-0.09</v>
@@ -1664,7 +1664,7 @@
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="B22">
         <v>12</v>
@@ -1683,10 +1683,10 @@
       </c>
       <c r="F22">
         <f t="shared" si="3"/>
-        <v>-8.3676000000000013</v>
+        <v>8.3676000000000013</v>
       </c>
       <c r="K22" s="7" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="L22" s="7">
         <v>-0.19</v>
@@ -1694,7 +1694,7 @@
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" s="7" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="B23">
         <v>13</v>
@@ -1713,10 +1713,10 @@
       </c>
       <c r="F23">
         <f t="shared" si="3"/>
-        <v>-6.2022999999999993</v>
+        <v>6.2022999999999993</v>
       </c>
       <c r="K23" s="7" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="L23" s="7">
         <v>-0.13</v>
@@ -1724,7 +1724,7 @@
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" s="7" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="B24">
         <v>14</v>
@@ -1743,10 +1743,10 @@
       </c>
       <c r="F24">
         <f t="shared" si="3"/>
-        <v>-2.0552000000000001</v>
+        <v>2.0552000000000001</v>
       </c>
       <c r="K24" s="7" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="L24" s="7">
         <v>-0.04</v>
@@ -1754,7 +1754,7 @@
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" s="7" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="B25">
         <v>15</v>
@@ -1773,10 +1773,10 @@
       </c>
       <c r="F25">
         <f t="shared" si="3"/>
-        <v>-22.02</v>
+        <v>22.02</v>
       </c>
       <c r="K25" s="7" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="L25" s="7">
         <v>-0.4</v>
@@ -1784,7 +1784,7 @@
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A26" s="7" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="B26">
         <v>16</v>
@@ -1803,10 +1803,10 @@
       </c>
       <c r="F26">
         <f t="shared" si="3"/>
-        <v>-5.2847999999999997</v>
+        <v>5.2847999999999997</v>
       </c>
       <c r="K26" s="7" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="L26" s="7">
         <v>-0.09</v>
@@ -1814,7 +1814,7 @@
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27" s="7" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="B27">
         <v>17</v>
@@ -1836,7 +1836,7 @@
         <v>0</v>
       </c>
       <c r="K27" s="7" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="L27" s="7">
         <v>0</v>
@@ -1844,7 +1844,7 @@
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" s="7" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="B28">
         <v>18</v>
@@ -1863,10 +1863,10 @@
       </c>
       <c r="F28">
         <f t="shared" si="3"/>
-        <v>-29.066399999999998</v>
+        <v>29.066399999999998</v>
       </c>
       <c r="K28" s="7" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="L28" s="7">
         <v>-0.44</v>
@@ -1874,7 +1874,7 @@
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A29" s="7" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="B29">
         <v>19</v>
@@ -1893,10 +1893,10 @@
       </c>
       <c r="F29">
         <f t="shared" si="3"/>
-        <v>-14.643299999999998</v>
+        <v>14.643299999999998</v>
       </c>
       <c r="K29" s="7" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="L29" s="7">
         <v>-0.21</v>
@@ -1904,7 +1904,7 @@
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A30" s="7" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="B30">
         <v>20</v>
@@ -1923,10 +1923,10 @@
       </c>
       <c r="F30">
         <f t="shared" si="3"/>
-        <v>-15.414</v>
+        <v>15.414</v>
       </c>
       <c r="K30" s="7" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="L30" s="7">
         <v>-0.21</v>
@@ -1934,7 +1934,7 @@
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="B31">
         <v>21</v>
@@ -1956,7 +1956,7 @@
         <v>0</v>
       </c>
       <c r="K31" s="7" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="L31" s="7">
         <v>0</v>
@@ -1964,7 +1964,7 @@
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A32" s="7" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="B32">
         <v>22</v>
@@ -1983,10 +1983,10 @@
       </c>
       <c r="F32">
         <f t="shared" si="3"/>
-        <v>-3.2296</v>
+        <v>3.2296</v>
       </c>
       <c r="K32" s="7" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="L32" s="7">
         <v>-0.04</v>
@@ -1994,7 +1994,7 @@
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A33" s="7" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="B33">
         <v>23</v>
@@ -2013,10 +2013,10 @@
       </c>
       <c r="F33">
         <f t="shared" si="3"/>
-        <v>-5.9087000000000005</v>
+        <v>5.9087000000000005</v>
       </c>
       <c r="K33" s="7" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="L33" s="7">
         <v>-7.0000000000000007E-2</v>
@@ -2024,7 +2024,7 @@
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A34" s="7" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="B34">
         <v>24</v>
@@ -2043,10 +2043,10 @@
       </c>
       <c r="F34">
         <f t="shared" si="3"/>
-        <v>-3.5231999999999997</v>
+        <v>3.5231999999999997</v>
       </c>
       <c r="K34" s="7" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="L34" s="7">
         <v>-0.04</v>
@@ -2054,7 +2054,7 @@
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A35" s="7" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="B35">
         <v>25</v>
@@ -2073,10 +2073,10 @@
       </c>
       <c r="F35">
         <f t="shared" si="3"/>
-        <v>-22.02</v>
+        <v>22.02</v>
       </c>
       <c r="K35" s="7" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="L35" s="7">
         <v>-0.24</v>
@@ -2084,7 +2084,7 @@
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A36" s="7" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="B36">
         <v>26</v>
@@ -2103,10 +2103,10 @@
       </c>
       <c r="F36">
         <f t="shared" si="3"/>
-        <v>-16.221399999999999</v>
+        <v>16.221399999999999</v>
       </c>
       <c r="K36" s="7" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="L36" s="7">
         <v>-0.17</v>
@@ -2114,7 +2114,7 @@
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A37" s="7" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="B37">
         <v>27</v>
@@ -2133,10 +2133,10 @@
       </c>
       <c r="F37">
         <f t="shared" si="3"/>
-        <v>-2.9726999999999997</v>
+        <v>2.9726999999999997</v>
       </c>
       <c r="K37" s="7" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="L37" s="7">
         <v>-0.03</v>
@@ -2144,7 +2144,7 @@
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A38" s="7" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="B38">
         <v>28</v>
@@ -2163,10 +2163,10 @@
       </c>
       <c r="F38">
         <f t="shared" si="3"/>
-        <v>-2.0552000000000001</v>
+        <v>2.0552000000000001</v>
       </c>
       <c r="K38" s="7" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="L38" s="7">
         <v>-0.02</v>
@@ -2174,7 +2174,7 @@
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A39" s="7" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="B39">
         <v>29</v>
@@ -2193,10 +2193,10 @@
       </c>
       <c r="F39">
         <f t="shared" si="3"/>
-        <v>-45.764900000000004</v>
+        <v>45.764900000000004</v>
       </c>
       <c r="K39" s="7" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="L39" s="7">
         <v>-0.43</v>
@@ -2204,7 +2204,7 @@
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A40" s="7" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="B40">
         <v>30</v>
@@ -2223,10 +2223,10 @@
       </c>
       <c r="F40">
         <f t="shared" si="3"/>
-        <v>-15.414</v>
+        <v>15.414</v>
       </c>
       <c r="K40" s="7" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="L40" s="7">
         <v>-0.14000000000000001</v>
@@ -2234,7 +2234,7 @@
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A41" s="7" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="B41">
         <v>31</v>
@@ -2256,7 +2256,7 @@
         <v>0</v>
       </c>
       <c r="K41" s="7" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="L41" s="7">
         <v>0</v>
@@ -2264,7 +2264,7 @@
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A42" s="7" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="B42">
         <v>32</v>
@@ -2283,10 +2283,10 @@
       </c>
       <c r="F42">
         <f t="shared" si="3"/>
-        <v>-14.092799999999999</v>
+        <v>14.092799999999999</v>
       </c>
       <c r="K42" s="7" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="L42" s="7">
         <v>-0.12</v>
@@ -2294,7 +2294,7 @@
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A43" s="7" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="B43">
         <v>33</v>
@@ -2313,10 +2313,10 @@
       </c>
       <c r="F43">
         <f t="shared" si="3"/>
-        <v>-15.744299999999999</v>
+        <v>15.744299999999999</v>
       </c>
       <c r="K43" s="7" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="L43" s="7">
         <v>-0.13</v>
@@ -2324,7 +2324,7 @@
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A44" s="7" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="B44">
         <v>34</v>
@@ -2343,10 +2343,10 @@
       </c>
       <c r="F44">
         <f t="shared" si="3"/>
-        <v>-19.9648</v>
+        <v>19.9648</v>
       </c>
       <c r="K44" s="7" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="L44" s="7">
         <v>-0.16</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A45" s="7" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="B45">
         <v>35</v>
@@ -2373,10 +2373,10 @@
       </c>
       <c r="F45">
         <f t="shared" si="3"/>
-        <v>-11.560499999999999</v>
+        <v>11.560499999999999</v>
       </c>
       <c r="K45" s="7" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="L45" s="7">
         <v>-0.09</v>
@@ -2384,7 +2384,7 @@
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A46" s="7" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="B46">
         <v>36</v>
@@ -2406,7 +2406,7 @@
         <v>0</v>
       </c>
       <c r="K46" s="7" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="L46" s="7">
         <v>0</v>
@@ -2414,7 +2414,7 @@
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A47" s="7" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="B47">
         <v>37</v>
@@ -2433,10 +2433,10 @@
       </c>
       <c r="F47">
         <f t="shared" si="3"/>
-        <v>-5.4315999999999995</v>
+        <v>5.4315999999999995</v>
       </c>
       <c r="K47" s="7" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="L47" s="7">
         <v>-0.04</v>
@@ -2444,7 +2444,7 @@
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A48" s="7" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="B48">
         <v>38</v>
@@ -2463,10 +2463,10 @@
       </c>
       <c r="F48">
         <f t="shared" si="3"/>
-        <v>-4.1837999999999997</v>
+        <v>4.1837999999999997</v>
       </c>
       <c r="K48" s="7" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="L48" s="7">
         <v>-0.03</v>
@@ -2474,7 +2474,7 @@
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A49" s="7" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="B49">
         <v>39</v>
@@ -2493,10 +2493,10 @@
       </c>
       <c r="F49">
         <f t="shared" si="3"/>
-        <v>-20.038200000000003</v>
+        <v>20.038200000000003</v>
       </c>
       <c r="K49" s="7" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="L49" s="7">
         <v>-0.14000000000000001</v>
@@ -2504,7 +2504,7 @@
     </row>
     <row r="50" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A50" s="7" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="B50">
         <v>40</v>
@@ -2523,10 +2523,10 @@
       </c>
       <c r="F50">
         <f t="shared" si="3"/>
-        <v>-45.508000000000003</v>
+        <v>45.508000000000003</v>
       </c>
       <c r="K50" s="7" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="L50" s="7">
         <v>-0.31</v>
@@ -2534,7 +2534,7 @@
     </row>
     <row r="51" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A51" s="7" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="B51">
         <v>41</v>
@@ -2553,10 +2553,10 @@
       </c>
       <c r="F51">
         <f t="shared" si="3"/>
-        <v>-34.6081</v>
+        <v>34.6081</v>
       </c>
       <c r="K51" s="7" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="L51" s="7">
         <v>-0.23</v>
@@ -2564,7 +2564,7 @@
     </row>
     <row r="52" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A52" s="7" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="B52">
         <v>42</v>
@@ -2583,10 +2583,10 @@
       </c>
       <c r="F52">
         <f t="shared" si="3"/>
-        <v>-26.203800000000001</v>
+        <v>26.203800000000001</v>
       </c>
       <c r="K52" s="7" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="L52" s="7">
         <v>-0.17</v>
@@ -2594,7 +2594,7 @@
     </row>
     <row r="53" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A53" s="7" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="B53">
         <v>43</v>
@@ -2613,10 +2613,10 @@
       </c>
       <c r="F53">
         <f t="shared" si="3"/>
-        <v>-26.8277</v>
+        <v>26.8277</v>
       </c>
       <c r="K53" s="7" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="L53" s="7">
         <v>-0.17</v>
@@ -2624,7 +2624,7 @@
     </row>
     <row r="54" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A54" s="7" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="B54">
         <v>44</v>
@@ -2643,10 +2643,10 @@
       </c>
       <c r="F54">
         <f t="shared" si="3"/>
-        <v>-12.9184</v>
+        <v>12.9184</v>
       </c>
       <c r="K54" s="7" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="L54" s="7">
         <v>-0.08</v>
@@ -2654,7 +2654,7 @@
     </row>
     <row r="55" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A55" s="7" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="B55">
         <v>45</v>
@@ -2673,10 +2673,10 @@
       </c>
       <c r="F55">
         <f t="shared" si="3"/>
-        <v>-18.166499999999999</v>
+        <v>18.166499999999999</v>
       </c>
       <c r="K55" s="7" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="L55" s="7">
         <v>-0.11</v>
@@ -2684,7 +2684,7 @@
     </row>
     <row r="56" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A56" s="7" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="B56">
         <v>46</v>
@@ -2706,7 +2706,7 @@
         <v>0</v>
       </c>
       <c r="K56" s="7" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="L56" s="7">
         <v>0</v>
@@ -2714,7 +2714,7 @@
     </row>
     <row r="57" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A57" s="7" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="B57">
         <v>47</v>
@@ -2733,10 +2733,10 @@
       </c>
       <c r="F57">
         <f t="shared" si="3"/>
-        <v>-3.4498000000000002</v>
+        <v>3.4498000000000002</v>
       </c>
       <c r="K57" s="7" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="L57" s="7">
         <v>-0.02</v>
@@ -2744,7 +2744,7 @@
     </row>
     <row r="58" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A58" s="7" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="B58">
         <v>48</v>
@@ -2763,10 +2763,10 @@
       </c>
       <c r="F58">
         <f t="shared" si="3"/>
-        <v>-14.092799999999999</v>
+        <v>14.092799999999999</v>
       </c>
       <c r="K58" s="7" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="L58" s="7">
         <v>-0.08</v>
@@ -2774,7 +2774,7 @@
     </row>
     <row r="59" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A59" s="7" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="B59">
         <v>49</v>
@@ -2793,10 +2793,10 @@
       </c>
       <c r="F59">
         <f t="shared" si="3"/>
-        <v>-10.7898</v>
+        <v>10.7898</v>
       </c>
       <c r="K59" s="7" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="L59" s="7">
         <v>-0.06</v>
@@ -2804,7 +2804,7 @@
     </row>
     <row r="60" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A60" s="7" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="B60">
         <v>50</v>
@@ -2823,10 +2823,10 @@
       </c>
       <c r="F60">
         <f t="shared" si="3"/>
-        <v>-22.02</v>
+        <v>22.02</v>
       </c>
       <c r="K60" s="7" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="L60" s="7">
         <v>-0.12</v>
@@ -2834,7 +2834,7 @@
     </row>
     <row r="61" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A61" s="7" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="B61">
         <v>51</v>
@@ -2853,10 +2853,10 @@
       </c>
       <c r="F61">
         <f t="shared" si="3"/>
-        <v>-13.101900000000001</v>
+        <v>13.101900000000001</v>
       </c>
       <c r="K61" s="7" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="L61" s="7">
         <v>-7.0000000000000007E-2</v>
@@ -2864,7 +2864,7 @@
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A62" s="7" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="B62">
         <v>52</v>
@@ -2883,10 +2883,10 @@
       </c>
       <c r="F62">
         <f t="shared" si="3"/>
-        <v>-24.809199999999997</v>
+        <v>24.809199999999997</v>
       </c>
       <c r="K62" s="7" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="L62" s="7">
         <v>-0.13</v>
@@ -2894,7 +2894,7 @@
     </row>
     <row r="63" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A63" s="7" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="B63">
         <v>53</v>
@@ -2916,7 +2916,7 @@
         <v>0</v>
       </c>
       <c r="K63" s="7" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="L63" s="7">
         <v>0</v>
@@ -2924,7 +2924,7 @@
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A64" s="7" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="B64">
         <v>54</v>
@@ -2943,10 +2943,10 @@
       </c>
       <c r="F64">
         <f t="shared" si="3"/>
-        <v>-47.563199999999995</v>
+        <v>47.563199999999995</v>
       </c>
       <c r="K64" s="7" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="L64" s="7">
         <v>-0.24</v>
@@ -2954,7 +2954,7 @@
     </row>
     <row r="65" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A65" s="7" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="B65">
         <v>55</v>
@@ -2973,10 +2973,10 @@
       </c>
       <c r="F65">
         <f t="shared" si="3"/>
-        <v>-64.591999999999999</v>
+        <v>64.591999999999999</v>
       </c>
       <c r="K65" s="7" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="L65" s="7">
         <v>-0.32</v>
@@ -2984,7 +2984,7 @@
     </row>
     <row r="66" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A66" s="7" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="B66">
         <v>56</v>
@@ -3006,7 +3006,7 @@
         <v>0</v>
       </c>
       <c r="K66" s="7" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="L66" s="7">
         <v>0</v>
@@ -3014,7 +3014,7 @@
     </row>
     <row r="67" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A67" s="7" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="B67">
         <v>57</v>
@@ -3036,7 +3036,7 @@
         <v>0</v>
       </c>
       <c r="K67" s="7" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="L67" s="7">
         <v>0</v>
@@ -3044,7 +3044,7 @@
     </row>
     <row r="68" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A68" s="7" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="B68">
         <v>58</v>
@@ -3063,10 +3063,10 @@
       </c>
       <c r="F68">
         <f t="shared" si="3"/>
-        <v>-21.286000000000001</v>
+        <v>21.286000000000001</v>
       </c>
       <c r="K68" s="7" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="L68" s="7">
         <v>-0.1</v>
@@ -3074,7 +3074,7 @@
     </row>
     <row r="69" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A69" s="7" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="B69">
         <v>59</v>
@@ -3093,10 +3093,10 @@
       </c>
       <c r="F69">
         <f t="shared" si="3"/>
-        <v>-71.454900000000009</v>
+        <v>71.454900000000009</v>
       </c>
       <c r="K69" s="7" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="L69" s="7">
         <v>-0.33</v>
@@ -3104,7 +3104,7 @@
     </row>
     <row r="70" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A70" s="7" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="B70">
         <v>60</v>
@@ -3126,7 +3126,7 @@
         <v>0</v>
       </c>
       <c r="K70" s="7" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="L70" s="7">
         <v>0</v>
@@ -3134,7 +3134,7 @@
     </row>
     <row r="71" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A71" s="7" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="B71">
         <v>61</v>
@@ -3153,10 +3153,10 @@
       </c>
       <c r="F71">
         <f t="shared" si="3"/>
-        <v>-11.1935</v>
+        <v>11.1935</v>
       </c>
       <c r="K71" s="7" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="L71" s="7">
         <v>-0.05</v>
@@ -3164,7 +3164,7 @@
     </row>
     <row r="72" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A72" s="7" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="B72">
         <v>62</v>
@@ -3183,10 +3183,10 @@
       </c>
       <c r="F72">
         <f t="shared" si="3"/>
-        <v>-59.160400000000003</v>
+        <v>59.160400000000003</v>
       </c>
       <c r="K72" s="7" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="L72" s="7">
         <v>-0.26</v>
@@ -3194,7 +3194,7 @@
     </row>
     <row r="73" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A73" s="7" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="B73">
         <v>63</v>
@@ -3213,10 +3213,10 @@
       </c>
       <c r="F73">
         <f t="shared" si="3"/>
-        <v>-60.114599999999996</v>
+        <v>60.114599999999996</v>
       </c>
       <c r="K73" s="7" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="L73" s="7">
         <v>-0.26</v>
@@ -3224,7 +3224,7 @@
     </row>
     <row r="74" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A74" s="7" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="B74">
         <v>64</v>
@@ -3243,10 +3243,10 @@
       </c>
       <c r="F74">
         <f t="shared" si="3"/>
-        <v>-7.0463999999999993</v>
+        <v>7.0463999999999993</v>
       </c>
       <c r="K74" s="7" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="L74" s="7">
         <v>-0.03</v>
@@ -3254,7 +3254,7 @@
     </row>
     <row r="75" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A75" s="7" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="B75">
         <v>65</v>
@@ -3273,10 +3273,10 @@
       </c>
       <c r="F75">
         <f t="shared" si="3"/>
-        <v>-88.263500000000008</v>
+        <v>88.263500000000008</v>
       </c>
       <c r="K75" s="7" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="L75" s="7">
         <v>-0.37</v>
@@ -3284,7 +3284,7 @@
     </row>
     <row r="76" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A76" s="7" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="B76">
         <v>66</v>
@@ -3302,11 +3302,11 @@
         <v>3.67</v>
       </c>
       <c r="F76">
-        <f t="shared" ref="F76:F94" si="7">D76*E76</f>
-        <v>-2.4222000000000001</v>
+        <f t="shared" ref="F76:F94" si="7">D76*E76*-1</f>
+        <v>2.4222000000000001</v>
       </c>
       <c r="K76" s="7" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="L76" s="7">
         <v>-0.01</v>
@@ -3314,7 +3314,7 @@
     </row>
     <row r="77" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A77" s="7" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="B77">
         <v>67</v>
@@ -3333,10 +3333,10 @@
       </c>
       <c r="F77">
         <f t="shared" si="7"/>
-        <v>-7.3766999999999987</v>
+        <v>7.3766999999999987</v>
       </c>
       <c r="K77" s="7" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="L77" s="7">
         <v>-0.03</v>
@@ -3344,7 +3344,7 @@
     </row>
     <row r="78" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A78" s="7" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="B78">
         <v>68</v>
@@ -3363,10 +3363,10 @@
       </c>
       <c r="F78">
         <f t="shared" si="7"/>
-        <v>-24.956000000000003</v>
+        <v>24.956000000000003</v>
       </c>
       <c r="K78" s="7" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="L78" s="7">
         <v>-0.1</v>
@@ -3374,7 +3374,7 @@
     </row>
     <row r="79" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A79" s="7" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="B79">
         <v>69</v>
@@ -3393,10 +3393,10 @@
       </c>
       <c r="F79">
         <f t="shared" si="7"/>
-        <v>-63.307499999999997</v>
+        <v>63.307499999999997</v>
       </c>
       <c r="K79" s="7" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="L79" s="7">
         <v>-0.25</v>
@@ -3404,7 +3404,7 @@
     </row>
     <row r="80" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A80" s="7" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="B80">
         <v>70</v>
@@ -3423,10 +3423,10 @@
       </c>
       <c r="F80">
         <f t="shared" si="7"/>
-        <v>-69.363</v>
+        <v>69.363</v>
       </c>
       <c r="K80" s="7" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="L80" s="7">
         <v>-0.27</v>
@@ -3434,7 +3434,7 @@
     </row>
     <row r="81" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A81" s="7" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="B81">
         <v>71</v>
@@ -3453,10 +3453,10 @@
       </c>
       <c r="F81">
         <f t="shared" si="7"/>
-        <v>-46.9026</v>
+        <v>46.9026</v>
       </c>
       <c r="K81" s="7" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="L81" s="7">
         <v>-0.18</v>
@@ -3464,7 +3464,7 @@
     </row>
     <row r="82" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A82" s="7" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="B82">
         <v>72</v>
@@ -3483,10 +3483,10 @@
       </c>
       <c r="F82">
         <f t="shared" si="7"/>
-        <v>-31.7088</v>
+        <v>31.7088</v>
       </c>
       <c r="K82" s="7" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="L82" s="7">
         <v>-0.12</v>
@@ -3494,7 +3494,7 @@
     </row>
     <row r="83" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A83" s="7" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="B83">
         <v>73</v>
@@ -3513,10 +3513,10 @@
       </c>
       <c r="F83">
         <f t="shared" si="7"/>
-        <v>-58.940199999999997</v>
+        <v>58.940199999999997</v>
       </c>
       <c r="K83" s="7" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="L83" s="7">
         <v>-0.22</v>
@@ -3524,7 +3524,7 @@
     </row>
     <row r="84" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A84" s="7" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="B84">
         <v>74</v>
@@ -3543,10 +3543,10 @@
       </c>
       <c r="F84">
         <f t="shared" si="7"/>
-        <v>-54.316000000000003</v>
+        <v>54.316000000000003</v>
       </c>
       <c r="K84" s="7" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="L84" s="7">
         <v>-0.2</v>
@@ -3554,7 +3554,7 @@
     </row>
     <row r="85" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A85" s="7" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="B85">
         <v>75</v>
@@ -3573,10 +3573,10 @@
       </c>
       <c r="F85">
         <f t="shared" si="7"/>
-        <v>-49.545000000000002</v>
+        <v>49.545000000000002</v>
       </c>
       <c r="K85" s="7" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="L85" s="7">
         <v>-0.18</v>
@@ -3584,7 +3584,7 @@
     </row>
     <row r="86" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A86" s="7" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="B86">
         <v>76</v>
@@ -3603,10 +3603,10 @@
       </c>
       <c r="F86">
         <f t="shared" si="7"/>
-        <v>-111.56800000000001</v>
+        <v>111.56800000000001</v>
       </c>
       <c r="K86" s="7" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="L86" s="7">
         <v>-0.4</v>
@@ -3614,7 +3614,7 @@
     </row>
     <row r="87" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A87" s="7" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="B87">
         <v>77</v>
@@ -3633,10 +3633,10 @@
       </c>
       <c r="F87">
         <f t="shared" si="7"/>
-        <v>-59.343899999999991</v>
+        <v>59.343899999999991</v>
       </c>
       <c r="K87" s="7" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="L87" s="7">
         <v>-0.21</v>
@@ -3644,7 +3644,7 @@
     </row>
     <row r="88" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A88" s="7" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B88">
         <v>78</v>
@@ -3663,10 +3663,10 @@
       </c>
       <c r="F88">
         <f t="shared" si="7"/>
-        <v>-111.6414</v>
+        <v>111.6414</v>
       </c>
       <c r="K88" s="7" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="L88" s="7">
         <v>-0.39</v>
@@ -3674,7 +3674,7 @@
     </row>
     <row r="89" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A89" s="7" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="B89">
         <v>79</v>
@@ -3693,10 +3693,10 @@
       </c>
       <c r="F89">
         <f t="shared" si="7"/>
-        <v>-200.05169999999998</v>
+        <v>200.05169999999998</v>
       </c>
       <c r="K89" s="7" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="L89" s="7">
         <v>-0.69</v>
@@ -3704,7 +3704,7 @@
     </row>
     <row r="90" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A90" s="7" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="B90">
         <v>80</v>
@@ -3726,7 +3726,7 @@
         <v>0</v>
       </c>
       <c r="K90" s="7" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="L90" s="7">
         <v>0</v>
@@ -3734,7 +3734,7 @@
     </row>
     <row r="91" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A91" s="7" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="B91">
         <v>81</v>
@@ -3753,10 +3753,10 @@
       </c>
       <c r="F91">
         <f t="shared" si="7"/>
-        <v>-20.808900000000001</v>
+        <v>20.808900000000001</v>
       </c>
       <c r="K91" s="7" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="L91" s="7">
         <v>-7.0000000000000007E-2</v>
@@ -3764,7 +3764,7 @@
     </row>
     <row r="92" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A92" s="7" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="B92">
         <v>82</v>
@@ -3783,10 +3783,10 @@
       </c>
       <c r="F92">
         <f t="shared" si="7"/>
-        <v>-171.53579999999997</v>
+        <v>171.53579999999997</v>
       </c>
       <c r="K92" s="7" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="L92" s="7">
         <v>-0.56999999999999995</v>
@@ -3794,7 +3794,7 @@
     </row>
     <row r="93" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A93" s="7" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="B93">
         <v>83</v>
@@ -3813,10 +3813,10 @@
       </c>
       <c r="F93">
         <f t="shared" si="7"/>
-        <v>-204.08870000000002</v>
+        <v>204.08870000000002</v>
       </c>
       <c r="K93" s="7" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="L93" s="7">
         <v>-0.67</v>
@@ -3824,7 +3824,7 @@
     </row>
     <row r="94" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A94" s="7" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="B94">
         <v>84</v>
@@ -3843,10 +3843,10 @@
       </c>
       <c r="F94">
         <f t="shared" si="7"/>
-        <v>-15.414</v>
+        <v>15.414</v>
       </c>
       <c r="K94" s="7" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="L94" s="7">
         <v>-0.05</v>
@@ -3864,7 +3864,7 @@
   <sheetData>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>131</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -3891,21 +3891,21 @@
         <v>24</v>
       </c>
       <c r="D8" t="s">
-        <v>130</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
-        <v>127</v>
+        <v>43</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>128</v>
+        <v>44</v>
       </c>
       <c r="C10" t="s">
         <v>23</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>129</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
feat(calculators): introduce land use activity input type field
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/16-lulucf/16-lulucf.xlsx
+++ b/packages/calculators/src/modules/test/16-lulucf/16-lulucf.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eddiesholl/Code/aginnovationaustralia/emissions-calculators/packages/calculators/src/modules/test/16-lulucf/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48E8A84F-F8F7-AB43-905E-4C39A8AD87BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{083C44B4-6804-0648-9E18-AA86D87208C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51220" yWindow="13240" windowWidth="28800" windowHeight="27420" activeTab="2" xr2:uid="{CC0FEAF9-C40F-694B-BCB9-117AFB86C05D}"/>
+    <workbookView xWindow="51200" yWindow="13240" windowWidth="28800" windowHeight="27420" activeTab="2" xr2:uid="{CC0FEAF9-C40F-694B-BCB9-117AFB86C05D}"/>
   </bookViews>
   <sheets>
     <sheet name="16.1.1.2" sheetId="1" r:id="rId1"/>

</xml_diff>